<commit_message>
docs: add guide of meanings of Eq, DC, CC, ASY in reference.xlsx
</commit_message>
<xml_diff>
--- a/reference.xlsx
+++ b/reference.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imagi\Documents\GitHub\hangul-overlap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{002DEF1D-A6EB-4EC1-809B-1A170BFDF3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5CFACA-DC2A-4D54-8174-D36987C16F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5244" yWindow="1704" windowWidth="20724" windowHeight="13548" xr2:uid="{44DA0D67-2440-4DBF-9106-819624DAECA4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="64">
   <si>
     <t>자음</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -277,6 +277,22 @@
   </si>
   <si>
     <t>ASY</t>
+  </si>
+  <si>
+    <t>Eq : Equal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DC : Double Consonants</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CC : Complex Consonants</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ASY : Asymmetric Vowels</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -484,7 +500,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -543,6 +559,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -887,232 +912,163 @@
   <sheetData>
     <row r="1" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45"/>
     <row r="2" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
+      <c r="Y2" s="22"/>
+    </row>
+    <row r="3" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="4" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="17" t="s">
+      <c r="R4" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="18"/>
-      <c r="T2" s="19"/>
-      <c r="W2" s="1" t="s">
+      <c r="S4" s="18"/>
+      <c r="T4" s="19"/>
+      <c r="W4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="X4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="Y4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="Z4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AA4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AB4" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AC4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AD2" s="3" t="s">
+      <c r="AD4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="AE2" s="3" t="s">
+      <c r="AE4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="AF2" s="3" t="s">
+      <c r="AF4" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AG2" s="3" t="s">
+      <c r="AG4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="AH2" s="3" t="s">
+      <c r="AH4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="AI2" s="3" t="s">
+      <c r="AI4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="AJ2" s="3" t="s">
+      <c r="AJ4" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="AK2" s="3" t="s">
+      <c r="AK4" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AL4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="AM2" s="3" t="s">
+      <c r="AM4" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="AN2" s="3" t="s">
+      <c r="AN4" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="AO2" s="3" t="s">
+      <c r="AO4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="AP2" s="3" t="s">
+      <c r="AP4" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="AQ2" s="3" t="s">
+      <c r="AQ4" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AR4" s="4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="5" t="s">
+    <row r="5" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="P3" s="6"/>
-      <c r="R3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="S3" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="T3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="W3" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AG3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AH3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR3" s="6"/>
-    </row>
-    <row r="4" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="P4" s="6"/>
-      <c r="R4" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="T4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="W4" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AA4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AH4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR4" s="6"/>
-    </row>
-    <row r="5" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -1124,7 +1080,7 @@
       <c r="H5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="O5" s="2" t="s">
@@ -1132,332 +1088,374 @@
       </c>
       <c r="P5" s="6"/>
       <c r="R5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="S5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="S5" s="8" t="s">
         <v>23</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="W5" s="10" t="s">
-        <v>40</v>
+        <v>18</v>
+      </c>
+      <c r="W5" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="AA5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="AR5" s="6"/>
     </row>
     <row r="6" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B6" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>58</v>
+        <v>16</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="P6" s="6"/>
       <c r="R6" s="7" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S6" s="5" t="s">
         <v>23</v>
       </c>
       <c r="T6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="W6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AH6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR6" s="6"/>
+    </row>
+    <row r="7" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P7" s="6"/>
+      <c r="R7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="W7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR7" s="6"/>
+    </row>
+    <row r="8" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P8" s="6"/>
+      <c r="R8" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="S8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="W6" s="10" t="s">
+      <c r="W8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="AA6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AR6" s="6"/>
-    </row>
-    <row r="7" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="5" t="s">
+      <c r="AA8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR8" s="6"/>
+    </row>
+    <row r="9" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B9" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="P7" s="6"/>
-      <c r="R7" s="11" t="s">
+      <c r="G9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P9" s="6"/>
+      <c r="R9" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="S7" s="12" t="s">
+      <c r="S9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="T7" s="13" t="s">
+      <c r="T9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="W7" s="10" t="s">
+      <c r="W9" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="Y7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA7" s="2" t="s">
+      <c r="Y9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AB7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AC7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AD7" s="2" t="s">
+      <c r="AB9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AE7" s="2" t="s">
+      <c r="AE9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AH7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AL7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR7" s="6"/>
-    </row>
-    <row r="8" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="5" t="s">
+      <c r="AH9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR9" s="6"/>
+    </row>
+    <row r="10" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="P8" s="6"/>
-      <c r="W8" s="10" t="s">
+      <c r="H10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P10" s="6"/>
+      <c r="W10" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="AC8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AE8" s="2" t="s">
+      <c r="AC10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE10" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AM8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR8" s="6"/>
-    </row>
-    <row r="9" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="5" t="s">
+      <c r="AM10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR10" s="6"/>
+    </row>
+    <row r="11" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="P9" s="6"/>
-      <c r="R9" s="17" t="s">
+      <c r="I11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P11" s="6"/>
+      <c r="R11" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="S9" s="18"/>
-      <c r="T9" s="18"/>
-      <c r="U9" s="19"/>
-      <c r="W9" s="10" t="s">
+      <c r="S11" s="18"/>
+      <c r="T11" s="18"/>
+      <c r="U11" s="19"/>
+      <c r="W11" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="AA9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AD9" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AE9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR9" s="6"/>
-    </row>
-    <row r="10" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="5" t="s">
+      <c r="AA11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR11" s="6"/>
+    </row>
+    <row r="12" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J10" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="P10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="R10" s="7" t="s">
+      <c r="J12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="R12" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="S10" s="2" t="s">
+      <c r="S12" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="T10" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="U10" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="W10" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE10" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AR10" s="6"/>
-    </row>
-    <row r="11" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="P11" s="6"/>
-      <c r="R11" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="S11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="T11" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="U11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="W11" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="AF11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AG11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AH11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AI11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AJ11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AR11" s="6"/>
-    </row>
-    <row r="12" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="P12" s="6"/>
-      <c r="R12" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="S12" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="T12" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG12" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AH12" s="2" t="s">
-        <v>16</v>
+        <v>45</v>
+      </c>
+      <c r="AE12" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="AR12" s="6"/>
     </row>
     <row r="13" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>58</v>
+        <v>9</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="P13" s="6"/>
       <c r="R13" s="7" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="T13" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="AF13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG13" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="AH13" s="2" t="s">
-        <v>58</v>
+        <v>16</v>
+      </c>
+      <c r="AI13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ13" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="AR13" s="6"/>
     </row>
     <row r="14" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="N14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L14" s="2" t="s">
         <v>58</v>
       </c>
       <c r="P14" s="6"/>
       <c r="R14" s="7" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="T14" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U14" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="AG14" s="2" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="AH14" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="AI14" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="AR14" s="6"/>
     </row>
     <row r="15" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B15" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="O15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>58</v>
       </c>
       <c r="P15" s="6"/>
@@ -1465,296 +1463,358 @@
         <v>4</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="T15" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH15" s="2" t="s">
         <v>58</v>
       </c>
       <c r="AR15" s="6"/>
     </row>
-    <row r="16" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="13" t="s">
-        <v>58</v>
-      </c>
+    <row r="16" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P16" s="6"/>
       <c r="R16" s="7" t="s">
         <v>4</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T16" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U16" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="AK16" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AL16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AN16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AO16" s="2" t="s">
-        <v>59</v>
+        <v>49</v>
+      </c>
+      <c r="AG16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI16" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="AR16" s="6"/>
     </row>
-    <row r="17" spans="18:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P17" s="6"/>
       <c r="R17" s="7" t="s">
         <v>4</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="T17" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U17" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AL17" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AM17" s="2" t="s">
-        <v>16</v>
+        <v>50</v>
+      </c>
+      <c r="AJ17" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="AR17" s="6"/>
     </row>
-    <row r="18" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B18" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="13" t="s">
+        <v>58</v>
+      </c>
       <c r="R18" s="7" t="s">
         <v>4</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="T18" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U18" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
+      </c>
+      <c r="AK18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL18" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="AM18" s="2" t="s">
-        <v>58</v>
+        <v>16</v>
+      </c>
+      <c r="AN18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO18" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="AR18" s="6"/>
     </row>
-    <row r="19" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
       <c r="R19" s="7" t="s">
         <v>4</v>
       </c>
       <c r="S19" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="T19" s="5" t="s">
         <v>36</v>
       </c>
       <c r="U19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="W19" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="AL19" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AM19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR19" s="6"/>
+    </row>
+    <row r="20" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R20" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="T20" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="U20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="W20" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM20" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR20" s="6"/>
+    </row>
+    <row r="21" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R21" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="T21" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="U21" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="W19" s="10" t="s">
+      <c r="W21" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="AL19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AN19" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AR19" s="6"/>
-    </row>
-    <row r="20" spans="18:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="R20" s="11" t="s">
+      <c r="AL21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN21" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR21" s="6"/>
+    </row>
+    <row r="22" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="R22" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="S20" s="14" t="s">
+      <c r="S22" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="T20" s="12" t="s">
+      <c r="T22" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="U20" s="13" t="s">
+      <c r="U22" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="W20" s="10" t="s">
+      <c r="W22" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="AO20" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AR20" s="6"/>
-    </row>
-    <row r="21" spans="18:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="W21" s="10" t="s">
+      <c r="AO22" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR22" s="6"/>
+    </row>
+    <row r="23" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="W23" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AF21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AG21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AH21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AI21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AJ21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AK21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AL21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AN21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AO21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AP21" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AQ21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR21" s="6"/>
-    </row>
-    <row r="22" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="W22" s="10" t="s">
+      <c r="AF23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AK23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP23" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR23" s="6"/>
+    </row>
+    <row r="24" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="W24" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AG22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AH22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AI22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AL22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AN22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AQ22" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AR22" s="6"/>
-    </row>
-    <row r="23" spans="18:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="W23" s="15" t="s">
+      <c r="AG24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AL24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ24" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR24" s="6"/>
+    </row>
+    <row r="25" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="W25" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="X23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AB23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AD23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AE23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AF23" s="14"/>
-      <c r="AG23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AH23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AI23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AJ23" s="14"/>
-      <c r="AK23" s="14"/>
-      <c r="AL23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AN23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AO23" s="14"/>
-      <c r="AP23" s="14"/>
-      <c r="AQ23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR23" s="13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="24" spans="18:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4"/>
-    <row r="27" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="X25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF25" s="14"/>
+      <c r="AG25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ25" s="14"/>
+      <c r="AK25" s="14"/>
+      <c r="AL25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO25" s="14"/>
+      <c r="AP25" s="14"/>
+      <c r="AQ25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="AR25" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4"/>
+    <row r="27" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="X27" s="16"/>
       <c r="Y27" s="16"/>
       <c r="Z27" s="16"/>
@@ -1776,7 +1836,7 @@
       <c r="AP27" s="16"/>
       <c r="AQ27" s="16"/>
     </row>
-    <row r="28" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="X28" s="16"/>
       <c r="Y28" s="16"/>
       <c r="Z28" s="16"/>
@@ -1798,7 +1858,7 @@
       <c r="AP28" s="16"/>
       <c r="AQ28" s="16"/>
     </row>
-    <row r="29" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="X29" s="16"/>
       <c r="Y29" s="16"/>
       <c r="Z29" s="16"/>
@@ -1820,7 +1880,7 @@
       <c r="AP29" s="16"/>
       <c r="AQ29" s="16"/>
     </row>
-    <row r="30" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="X30" s="16"/>
       <c r="Y30" s="16"/>
       <c r="Z30" s="16"/>
@@ -1842,7 +1902,7 @@
       <c r="AP30" s="16"/>
       <c r="AQ30" s="16"/>
     </row>
-    <row r="31" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="X31" s="16"/>
       <c r="Y31" s="16"/>
       <c r="Z31" s="16"/>
@@ -1864,7 +1924,7 @@
       <c r="AP31" s="16"/>
       <c r="AQ31" s="16"/>
     </row>
-    <row r="32" spans="18:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="X32" s="16"/>
       <c r="Y32" s="16"/>
       <c r="Z32" s="16"/>
@@ -2217,9 +2277,13 @@
       <c r="AQ47" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="R2:T2"/>
-    <mergeCell ref="R9:U9"/>
+  <mergeCells count="6">
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="R11:U11"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:K2"/>
+    <mergeCell ref="L2:R2"/>
+    <mergeCell ref="S2:Y2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: missing overlap relations between DC/CCs
</commit_message>
<xml_diff>
--- a/reference.xlsx
+++ b/reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imagi\Documents\GitHub\hangul-overlap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5CFACA-DC2A-4D54-8174-D36987C16F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B13B4F7-DA26-4AF4-9CDC-EF93CA61098C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5244" yWindow="1704" windowWidth="20724" windowHeight="13548" xr2:uid="{44DA0D67-2440-4DBF-9106-819624DAECA4}"/>
+    <workbookView xWindow="7248" yWindow="2292" windowWidth="20724" windowHeight="13548" xr2:uid="{44DA0D67-2440-4DBF-9106-819624DAECA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="65">
   <si>
     <t>자음</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -292,6 +292,10 @@
   </si>
   <si>
     <t>ASY : Asymmetric Vowels</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>쌍자음/겹받침 간 관계는 두 자음이 모두 성립할 시 성립</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -561,13 +565,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -944,6 +948,22 @@
       <c r="W2" s="21"/>
       <c r="X2" s="21"/>
       <c r="Y2" s="22"/>
+      <c r="AA2" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB2" s="21"/>
+      <c r="AC2" s="21"/>
+      <c r="AD2" s="21"/>
+      <c r="AE2" s="21"/>
+      <c r="AF2" s="21"/>
+      <c r="AG2" s="21"/>
+      <c r="AH2" s="21"/>
+      <c r="AI2" s="21"/>
+      <c r="AJ2" s="21"/>
+      <c r="AK2" s="21"/>
+      <c r="AL2" s="21"/>
+      <c r="AM2" s="21"/>
+      <c r="AN2" s="22"/>
     </row>
     <row r="3" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="2:44" ht="19.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
@@ -1756,6 +1776,22 @@
       <c r="AR24" s="6"/>
     </row>
     <row r="25" spans="2:44" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="C25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="16"/>
+      <c r="N25" s="16"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="16"/>
       <c r="W25" s="15" t="s">
         <v>57</v>
       </c>
@@ -1813,8 +1849,41 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4"/>
+    <row r="26" spans="2:44" ht="19.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="C26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="16"/>
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="16"/>
+    </row>
     <row r="27" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="16"/>
       <c r="X27" s="16"/>
       <c r="Y27" s="16"/>
       <c r="Z27" s="16"/>
@@ -1837,6 +1906,22 @@
       <c r="AQ27" s="16"/>
     </row>
     <row r="28" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="16"/>
       <c r="X28" s="16"/>
       <c r="Y28" s="16"/>
       <c r="Z28" s="16"/>
@@ -1859,21 +1944,22 @@
       <c r="AQ28" s="16"/>
     </row>
     <row r="29" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="X29" s="16"/>
-      <c r="Y29" s="16"/>
-      <c r="Z29" s="16"/>
-      <c r="AA29" s="16"/>
-      <c r="AB29" s="16"/>
-      <c r="AC29" s="16"/>
-      <c r="AD29" s="16"/>
-      <c r="AE29" s="16"/>
-      <c r="AF29" s="16"/>
-      <c r="AG29" s="16"/>
-      <c r="AH29" s="16"/>
-      <c r="AI29" s="16"/>
-      <c r="AJ29" s="16"/>
-      <c r="AK29" s="16"/>
-      <c r="AL29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="16"/>
+      <c r="N29" s="16"/>
+      <c r="O29" s="16"/>
+      <c r="P29" s="16"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
+      <c r="S29" s="16"/>
       <c r="AM29" s="16"/>
       <c r="AN29" s="16"/>
       <c r="AO29" s="16"/>
@@ -1881,6 +1967,22 @@
       <c r="AQ29" s="16"/>
     </row>
     <row r="30" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="16"/>
+      <c r="N30" s="16"/>
+      <c r="O30" s="16"/>
+      <c r="P30" s="16"/>
+      <c r="Q30" s="16"/>
+      <c r="R30" s="16"/>
+      <c r="S30" s="16"/>
       <c r="X30" s="16"/>
       <c r="Y30" s="16"/>
       <c r="Z30" s="16"/>
@@ -1903,6 +2005,22 @@
       <c r="AQ30" s="16"/>
     </row>
     <row r="31" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
+      <c r="M31" s="16"/>
+      <c r="N31" s="16"/>
+      <c r="O31" s="16"/>
+      <c r="P31" s="16"/>
+      <c r="Q31" s="16"/>
+      <c r="R31" s="16"/>
+      <c r="S31" s="16"/>
       <c r="X31" s="16"/>
       <c r="Y31" s="16"/>
       <c r="Z31" s="16"/>
@@ -1925,9 +2043,6 @@
       <c r="AQ31" s="16"/>
     </row>
     <row r="32" spans="2:44" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="X32" s="16"/>
-      <c r="Y32" s="16"/>
-      <c r="Z32" s="16"/>
       <c r="AA32" s="16"/>
       <c r="AB32" s="16"/>
       <c r="AC32" s="16"/>
@@ -1946,7 +2061,27 @@
       <c r="AP32" s="16"/>
       <c r="AQ32" s="16"/>
     </row>
-    <row r="33" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="16"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="16"/>
+      <c r="L33" s="16"/>
+      <c r="M33" s="16"/>
+      <c r="N33" s="16"/>
+      <c r="O33" s="16"/>
+      <c r="P33" s="16"/>
+      <c r="Q33" s="16"/>
+      <c r="R33" s="16"/>
+      <c r="S33" s="16"/>
+      <c r="T33" s="16"/>
+      <c r="U33" s="16"/>
+      <c r="V33" s="16"/>
+      <c r="W33" s="16"/>
       <c r="X33" s="16"/>
       <c r="Y33" s="16"/>
       <c r="Z33" s="16"/>
@@ -1968,7 +2103,27 @@
       <c r="AP33" s="16"/>
       <c r="AQ33" s="16"/>
     </row>
-    <row r="34" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="16"/>
+      <c r="L34" s="16"/>
+      <c r="M34" s="16"/>
+      <c r="N34" s="16"/>
+      <c r="O34" s="16"/>
+      <c r="P34" s="16"/>
+      <c r="Q34" s="16"/>
+      <c r="R34" s="16"/>
+      <c r="S34" s="16"/>
+      <c r="T34" s="16"/>
+      <c r="U34" s="16"/>
+      <c r="V34" s="16"/>
+      <c r="W34" s="16"/>
       <c r="X34" s="16"/>
       <c r="Y34" s="16"/>
       <c r="Z34" s="16"/>
@@ -1990,7 +2145,27 @@
       <c r="AP34" s="16"/>
       <c r="AQ34" s="16"/>
     </row>
-    <row r="35" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16"/>
+      <c r="O35" s="16"/>
+      <c r="P35" s="16"/>
+      <c r="Q35" s="16"/>
+      <c r="R35" s="16"/>
+      <c r="S35" s="16"/>
+      <c r="T35" s="16"/>
+      <c r="U35" s="16"/>
+      <c r="V35" s="16"/>
+      <c r="W35" s="16"/>
       <c r="X35" s="16"/>
       <c r="Y35" s="16"/>
       <c r="Z35" s="16"/>
@@ -2012,7 +2187,27 @@
       <c r="AP35" s="16"/>
       <c r="AQ35" s="16"/>
     </row>
-    <row r="36" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+      <c r="L36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="16"/>
+      <c r="O36" s="16"/>
+      <c r="P36" s="16"/>
+      <c r="Q36" s="16"/>
+      <c r="R36" s="16"/>
+      <c r="S36" s="16"/>
+      <c r="T36" s="16"/>
+      <c r="U36" s="16"/>
+      <c r="V36" s="16"/>
+      <c r="W36" s="16"/>
       <c r="X36" s="16"/>
       <c r="Y36" s="16"/>
       <c r="Z36" s="16"/>
@@ -2034,7 +2229,27 @@
       <c r="AP36" s="16"/>
       <c r="AQ36" s="16"/>
     </row>
-    <row r="37" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+      <c r="L37" s="16"/>
+      <c r="M37" s="16"/>
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="16"/>
+      <c r="S37" s="16"/>
+      <c r="T37" s="16"/>
+      <c r="U37" s="16"/>
+      <c r="V37" s="16"/>
+      <c r="W37" s="16"/>
       <c r="X37" s="16"/>
       <c r="Y37" s="16"/>
       <c r="Z37" s="16"/>
@@ -2056,7 +2271,27 @@
       <c r="AP37" s="16"/>
       <c r="AQ37" s="16"/>
     </row>
-    <row r="38" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="16"/>
+      <c r="L38" s="16"/>
+      <c r="M38" s="16"/>
+      <c r="N38" s="16"/>
+      <c r="O38" s="16"/>
+      <c r="P38" s="16"/>
+      <c r="Q38" s="16"/>
+      <c r="R38" s="16"/>
+      <c r="S38" s="16"/>
+      <c r="T38" s="16"/>
+      <c r="U38" s="16"/>
+      <c r="V38" s="16"/>
+      <c r="W38" s="16"/>
       <c r="X38" s="16"/>
       <c r="Y38" s="16"/>
       <c r="Z38" s="16"/>
@@ -2078,7 +2313,27 @@
       <c r="AP38" s="16"/>
       <c r="AQ38" s="16"/>
     </row>
-    <row r="39" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
+      <c r="L39" s="16"/>
+      <c r="M39" s="16"/>
+      <c r="N39" s="16"/>
+      <c r="O39" s="16"/>
+      <c r="P39" s="16"/>
+      <c r="Q39" s="16"/>
+      <c r="R39" s="16"/>
+      <c r="S39" s="16"/>
+      <c r="T39" s="16"/>
+      <c r="U39" s="16"/>
+      <c r="V39" s="16"/>
+      <c r="W39" s="16"/>
       <c r="X39" s="16"/>
       <c r="Y39" s="16"/>
       <c r="Z39" s="16"/>
@@ -2100,7 +2355,27 @@
       <c r="AP39" s="16"/>
       <c r="AQ39" s="16"/>
     </row>
-    <row r="40" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
+      <c r="S40" s="16"/>
+      <c r="T40" s="16"/>
+      <c r="U40" s="16"/>
+      <c r="V40" s="16"/>
+      <c r="W40" s="16"/>
       <c r="X40" s="16"/>
       <c r="Y40" s="16"/>
       <c r="Z40" s="16"/>
@@ -2122,7 +2397,27 @@
       <c r="AP40" s="16"/>
       <c r="AQ40" s="16"/>
     </row>
-    <row r="41" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="16"/>
+      <c r="G41" s="16"/>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="16"/>
+      <c r="L41" s="16"/>
+      <c r="M41" s="16"/>
+      <c r="N41" s="16"/>
+      <c r="O41" s="16"/>
+      <c r="P41" s="16"/>
+      <c r="Q41" s="16"/>
+      <c r="R41" s="16"/>
+      <c r="S41" s="16"/>
+      <c r="T41" s="16"/>
+      <c r="U41" s="16"/>
+      <c r="V41" s="16"/>
+      <c r="W41" s="16"/>
       <c r="X41" s="16"/>
       <c r="Y41" s="16"/>
       <c r="Z41" s="16"/>
@@ -2144,7 +2439,27 @@
       <c r="AP41" s="16"/>
       <c r="AQ41" s="16"/>
     </row>
-    <row r="42" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="16"/>
+      <c r="G42" s="16"/>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16"/>
+      <c r="J42" s="16"/>
+      <c r="L42" s="16"/>
+      <c r="M42" s="16"/>
+      <c r="N42" s="16"/>
+      <c r="O42" s="16"/>
+      <c r="P42" s="16"/>
+      <c r="Q42" s="16"/>
+      <c r="R42" s="16"/>
+      <c r="S42" s="16"/>
+      <c r="T42" s="16"/>
+      <c r="U42" s="16"/>
+      <c r="V42" s="16"/>
+      <c r="W42" s="16"/>
       <c r="X42" s="16"/>
       <c r="Y42" s="16"/>
       <c r="Z42" s="16"/>
@@ -2166,7 +2481,27 @@
       <c r="AP42" s="16"/>
       <c r="AQ42" s="16"/>
     </row>
-    <row r="43" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="16"/>
+      <c r="H43" s="16"/>
+      <c r="I43" s="16"/>
+      <c r="J43" s="16"/>
+      <c r="L43" s="16"/>
+      <c r="M43" s="16"/>
+      <c r="N43" s="16"/>
+      <c r="O43" s="16"/>
+      <c r="P43" s="16"/>
+      <c r="Q43" s="16"/>
+      <c r="R43" s="16"/>
+      <c r="S43" s="16"/>
+      <c r="T43" s="16"/>
+      <c r="U43" s="16"/>
+      <c r="V43" s="16"/>
+      <c r="W43" s="16"/>
       <c r="X43" s="16"/>
       <c r="Y43" s="16"/>
       <c r="Z43" s="16"/>
@@ -2188,7 +2523,27 @@
       <c r="AP43" s="16"/>
       <c r="AQ43" s="16"/>
     </row>
-    <row r="44" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="F44" s="16"/>
+      <c r="G44" s="16"/>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="16"/>
+      <c r="L44" s="16"/>
+      <c r="M44" s="16"/>
+      <c r="N44" s="16"/>
+      <c r="O44" s="16"/>
+      <c r="P44" s="16"/>
+      <c r="Q44" s="16"/>
+      <c r="R44" s="16"/>
+      <c r="S44" s="16"/>
+      <c r="T44" s="16"/>
+      <c r="U44" s="16"/>
+      <c r="V44" s="16"/>
+      <c r="W44" s="16"/>
       <c r="X44" s="16"/>
       <c r="Y44" s="16"/>
       <c r="Z44" s="16"/>
@@ -2210,7 +2565,27 @@
       <c r="AP44" s="16"/>
       <c r="AQ44" s="16"/>
     </row>
-    <row r="45" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="16"/>
+      <c r="H45" s="16"/>
+      <c r="I45" s="16"/>
+      <c r="J45" s="16"/>
+      <c r="L45" s="16"/>
+      <c r="M45" s="16"/>
+      <c r="N45" s="16"/>
+      <c r="O45" s="16"/>
+      <c r="P45" s="16"/>
+      <c r="Q45" s="16"/>
+      <c r="R45" s="16"/>
+      <c r="S45" s="16"/>
+      <c r="T45" s="16"/>
+      <c r="U45" s="16"/>
+      <c r="V45" s="16"/>
+      <c r="W45" s="16"/>
       <c r="X45" s="16"/>
       <c r="Y45" s="16"/>
       <c r="Z45" s="16"/>
@@ -2232,7 +2607,27 @@
       <c r="AP45" s="16"/>
       <c r="AQ45" s="16"/>
     </row>
-    <row r="46" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="16"/>
+      <c r="G46" s="16"/>
+      <c r="H46" s="16"/>
+      <c r="I46" s="16"/>
+      <c r="J46" s="16"/>
+      <c r="L46" s="16"/>
+      <c r="M46" s="16"/>
+      <c r="N46" s="16"/>
+      <c r="O46" s="16"/>
+      <c r="P46" s="16"/>
+      <c r="Q46" s="16"/>
+      <c r="R46" s="16"/>
+      <c r="S46" s="16"/>
+      <c r="T46" s="16"/>
+      <c r="U46" s="16"/>
+      <c r="V46" s="16"/>
+      <c r="W46" s="16"/>
       <c r="X46" s="16"/>
       <c r="Y46" s="16"/>
       <c r="Z46" s="16"/>
@@ -2254,7 +2649,27 @@
       <c r="AP46" s="16"/>
       <c r="AQ46" s="16"/>
     </row>
-    <row r="47" spans="24:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="3:43" ht="19.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="16"/>
+      <c r="L47" s="16"/>
+      <c r="M47" s="16"/>
+      <c r="N47" s="16"/>
+      <c r="O47" s="16"/>
+      <c r="P47" s="16"/>
+      <c r="Q47" s="16"/>
+      <c r="R47" s="16"/>
+      <c r="S47" s="16"/>
+      <c r="T47" s="16"/>
+      <c r="U47" s="16"/>
+      <c r="V47" s="16"/>
+      <c r="W47" s="16"/>
       <c r="X47" s="16"/>
       <c r="Y47" s="16"/>
       <c r="Z47" s="16"/>
@@ -2277,7 +2692,8 @@
       <c r="AQ47" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="AA2:AN2"/>
     <mergeCell ref="R4:T4"/>
     <mergeCell ref="R11:U11"/>
     <mergeCell ref="B2:D2"/>

</xml_diff>